<commit_message>
feat: add 37 head office departments/centers units and admin accounts
</commit_message>
<xml_diff>
--- a/exports/Danh_sach_tai_khoan_Agribank.xlsx
+++ b/exports/Danh_sach_tai_khoan_Agribank.xlsx
@@ -397,17 +397,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I158"/>
+  <dimension ref="A1:I195"/>
   <cols>
-    <col min="1" max="1" width="6.83203125" customWidth="1"/>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="35.83203125" customWidth="1"/>
     <col min="4" max="4" width="35.83203125" customWidth="1"/>
     <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="38.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="40.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="35.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="35.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4992,9 +4992,1082 @@
         <v>Tài khoản kê khai &amp; lập nhu cầu</v>
       </c>
     </row>
+    <row r="159">
+      <c r="A159">
+        <v>158</v>
+      </c>
+      <c r="B159" t="str">
+        <v>105060</v>
+      </c>
+      <c r="C159" t="str">
+        <v>UB Chính sách</v>
+      </c>
+      <c r="D159" t="str">
+        <v>UB Chính sách</v>
+      </c>
+      <c r="E159" t="str">
+        <v>105060_Admin</v>
+      </c>
+      <c r="F159" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G159" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H159" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I159" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160">
+        <v>159</v>
+      </c>
+      <c r="B160" t="str">
+        <v>105077</v>
+      </c>
+      <c r="C160" t="str">
+        <v>TT Chăm sóc KH</v>
+      </c>
+      <c r="D160" t="str">
+        <v>TT Chăm sóc KH</v>
+      </c>
+      <c r="E160" t="str">
+        <v>105077_Admin</v>
+      </c>
+      <c r="F160" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G160" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H160" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I160" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161">
+        <v>160</v>
+      </c>
+      <c r="B161" t="str">
+        <v>105052</v>
+      </c>
+      <c r="C161" t="str">
+        <v>Ban Định chế TC</v>
+      </c>
+      <c r="D161" t="str">
+        <v>Ban Định chế TC</v>
+      </c>
+      <c r="E161" t="str">
+        <v>105052_Admin</v>
+      </c>
+      <c r="F161" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G161" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H161" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I161" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162">
+        <v>161</v>
+      </c>
+      <c r="B162" t="str">
+        <v>1040</v>
+      </c>
+      <c r="C162" t="str">
+        <v>Trường Đào tạo CB</v>
+      </c>
+      <c r="D162" t="str">
+        <v>Trường Đào tạo CB</v>
+      </c>
+      <c r="E162" t="str">
+        <v>1040_Admin</v>
+      </c>
+      <c r="F162" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G162" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H162" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I162" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163">
+        <v>162</v>
+      </c>
+      <c r="B163" t="str">
+        <v>105066</v>
+      </c>
+      <c r="C163" t="str">
+        <v>Ban TCKT</v>
+      </c>
+      <c r="D163" t="str">
+        <v>Ban TCKT</v>
+      </c>
+      <c r="E163" t="str">
+        <v>105066_Admin</v>
+      </c>
+      <c r="F163" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G163" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H163" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I163" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164">
+        <v>163</v>
+      </c>
+      <c r="B164" t="str">
+        <v>105025</v>
+      </c>
+      <c r="C164" t="str">
+        <v>TTPD TD tại HCM</v>
+      </c>
+      <c r="D164" t="str">
+        <v>TTPD TD tại HCM</v>
+      </c>
+      <c r="E164" t="str">
+        <v>105025_Admin</v>
+      </c>
+      <c r="F164" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G164" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H164" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I164" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165">
+        <v>164</v>
+      </c>
+      <c r="B165" t="str">
+        <v>105047</v>
+      </c>
+      <c r="C165" t="str">
+        <v>TT DV &amp; Kiều hối</v>
+      </c>
+      <c r="D165" t="str">
+        <v>TT DV &amp; Kiều hối</v>
+      </c>
+      <c r="E165" t="str">
+        <v>105047_Admin</v>
+      </c>
+      <c r="F165" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G165" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H165" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I165" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166">
+        <v>165</v>
+      </c>
+      <c r="B166" t="str">
+        <v>105019</v>
+      </c>
+      <c r="C166" t="str">
+        <v>Ban Đầu tư</v>
+      </c>
+      <c r="D166" t="str">
+        <v>Ban Đầu tư</v>
+      </c>
+      <c r="E166" t="str">
+        <v>105019_Admin</v>
+      </c>
+      <c r="F166" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G166" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H166" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I166" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167">
+        <v>166</v>
+      </c>
+      <c r="B167" t="str">
+        <v>105024</v>
+      </c>
+      <c r="C167" t="str">
+        <v>TT thanh toán</v>
+      </c>
+      <c r="D167" t="str">
+        <v>TT thanh toán</v>
+      </c>
+      <c r="E167" t="str">
+        <v>105024_Admin</v>
+      </c>
+      <c r="F167" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G167" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H167" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I167" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168">
+        <v>167</v>
+      </c>
+      <c r="B168" t="str">
+        <v>105007</v>
+      </c>
+      <c r="C168" t="str">
+        <v>Ban TG Đảng Ủy</v>
+      </c>
+      <c r="D168" t="str">
+        <v>Ban TG Đảng Ủy</v>
+      </c>
+      <c r="E168" t="str">
+        <v>105007_Admin</v>
+      </c>
+      <c r="F168" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G168" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H168" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I168" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169">
+        <v>168</v>
+      </c>
+      <c r="B169" t="str">
+        <v>105009</v>
+      </c>
+      <c r="C169" t="str">
+        <v>Ban KT, GSNB</v>
+      </c>
+      <c r="D169" t="str">
+        <v>Ban KT, GSNB</v>
+      </c>
+      <c r="E169" t="str">
+        <v>105009_Admin</v>
+      </c>
+      <c r="F169" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G169" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H169" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I169" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170">
+        <v>169</v>
+      </c>
+      <c r="B170" t="str">
+        <v>105012</v>
+      </c>
+      <c r="C170" t="str">
+        <v>VP Đảng Ủy</v>
+      </c>
+      <c r="D170" t="str">
+        <v>VP Đảng Ủy</v>
+      </c>
+      <c r="E170" t="str">
+        <v>105012_Admin</v>
+      </c>
+      <c r="F170" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G170" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H170" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I170" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171">
+        <v>170</v>
+      </c>
+      <c r="B171" t="str">
+        <v>105010</v>
+      </c>
+      <c r="C171" t="str">
+        <v>BQLTS nợ-TS có</v>
+      </c>
+      <c r="D171" t="str">
+        <v>BQLTS nợ-TS có</v>
+      </c>
+      <c r="E171" t="str">
+        <v>105010_Admin</v>
+      </c>
+      <c r="F171" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G171" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H171" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I171" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172">
+        <v>171</v>
+      </c>
+      <c r="B172" t="str">
+        <v>105099</v>
+      </c>
+      <c r="C172" t="str">
+        <v>Ban KHDN</v>
+      </c>
+      <c r="D172" t="str">
+        <v>Ban KHDN</v>
+      </c>
+      <c r="E172" t="str">
+        <v>105099_Admin</v>
+      </c>
+      <c r="F172" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G172" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H172" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I172" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173">
+        <v>172</v>
+      </c>
+      <c r="B173" t="str">
+        <v>105029</v>
+      </c>
+      <c r="C173" t="str">
+        <v>VP Công đoàn</v>
+      </c>
+      <c r="D173" t="str">
+        <v>VP Công đoàn</v>
+      </c>
+      <c r="E173" t="str">
+        <v>105029_Admin</v>
+      </c>
+      <c r="F173" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G173" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H173" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I173" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174">
+        <v>173</v>
+      </c>
+      <c r="B174" t="str">
+        <v>105067</v>
+      </c>
+      <c r="C174" t="str">
+        <v>TT QLRR tín dụng</v>
+      </c>
+      <c r="D174" t="str">
+        <v>TT QLRR tín dụng</v>
+      </c>
+      <c r="E174" t="str">
+        <v>105067_Admin</v>
+      </c>
+      <c r="F174" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G174" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H174" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I174" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175">
+        <v>174</v>
+      </c>
+      <c r="B175" t="str">
+        <v>105013</v>
+      </c>
+      <c r="C175" t="str">
+        <v>Ban KH Chiến lược</v>
+      </c>
+      <c r="D175" t="str">
+        <v>Ban KH Chiến lược</v>
+      </c>
+      <c r="E175" t="str">
+        <v>105013_Admin</v>
+      </c>
+      <c r="F175" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G175" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H175" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I175" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176">
+        <v>175</v>
+      </c>
+      <c r="B176" t="str">
+        <v>1030</v>
+      </c>
+      <c r="C176" t="str">
+        <v>Trung tâm thẻ</v>
+      </c>
+      <c r="D176" t="str">
+        <v>Trung tâm thẻ</v>
+      </c>
+      <c r="E176" t="str">
+        <v>1030_Admin</v>
+      </c>
+      <c r="F176" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G176" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H176" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I176" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177">
+        <v>176</v>
+      </c>
+      <c r="B177" t="str">
+        <v>105073</v>
+      </c>
+      <c r="C177" t="str">
+        <v>BTĐ, phê duyệt TD</v>
+      </c>
+      <c r="D177" t="str">
+        <v>BTĐ, phê duyệt TD</v>
+      </c>
+      <c r="E177" t="str">
+        <v>105073_Admin</v>
+      </c>
+      <c r="F177" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G177" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H177" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I177" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178">
+        <v>177</v>
+      </c>
+      <c r="B178" t="str">
+        <v>105074</v>
+      </c>
+      <c r="C178" t="str">
+        <v>Ban CSTD</v>
+      </c>
+      <c r="D178" t="str">
+        <v>Ban CSTD</v>
+      </c>
+      <c r="E178" t="str">
+        <v>105074_Admin</v>
+      </c>
+      <c r="F178" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G178" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H178" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I178" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179">
+        <v>178</v>
+      </c>
+      <c r="B179" t="str">
+        <v>105011</v>
+      </c>
+      <c r="C179" t="str">
+        <v>Ban KHCN</v>
+      </c>
+      <c r="D179" t="str">
+        <v>Ban KHCN</v>
+      </c>
+      <c r="E179" t="str">
+        <v>105011_Admin</v>
+      </c>
+      <c r="F179" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G179" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H179" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I179" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180">
+        <v>179</v>
+      </c>
+      <c r="B180" t="str">
+        <v>1070</v>
+      </c>
+      <c r="C180" t="str">
+        <v>VPĐD Miền Nam</v>
+      </c>
+      <c r="D180" t="str">
+        <v>VPĐD Miền Nam</v>
+      </c>
+      <c r="E180" t="str">
+        <v>1070_Admin</v>
+      </c>
+      <c r="F180" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G180" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H180" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I180" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181">
+        <v>180</v>
+      </c>
+      <c r="B181" t="str">
+        <v>105038</v>
+      </c>
+      <c r="C181" t="str">
+        <v>UB QLRR</v>
+      </c>
+      <c r="D181" t="str">
+        <v>UB QLRR</v>
+      </c>
+      <c r="E181" t="str">
+        <v>105038_Admin</v>
+      </c>
+      <c r="F181" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G181" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H181" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I181" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182">
+        <v>181</v>
+      </c>
+      <c r="B182" t="str">
+        <v>105036</v>
+      </c>
+      <c r="C182" t="str">
+        <v>TT QLN có VĐ</v>
+      </c>
+      <c r="D182" t="str">
+        <v>TT QLN có VĐ</v>
+      </c>
+      <c r="E182" t="str">
+        <v>105036_Admin</v>
+      </c>
+      <c r="F182" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G182" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H182" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I182" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183">
+        <v>182</v>
+      </c>
+      <c r="B183" t="str">
+        <v>105048</v>
+      </c>
+      <c r="C183" t="str">
+        <v>Ban Tổ chức NS</v>
+      </c>
+      <c r="D183" t="str">
+        <v>Ban Tổ chức NS</v>
+      </c>
+      <c r="E183" t="str">
+        <v>105048_Admin</v>
+      </c>
+      <c r="F183" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G183" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H183" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I183" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184">
+        <v>183</v>
+      </c>
+      <c r="B184" t="str">
+        <v>105070</v>
+      </c>
+      <c r="C184" t="str">
+        <v>TTKD vốn, Tiền tệ</v>
+      </c>
+      <c r="D184" t="str">
+        <v>TTKD vốn, Tiền tệ</v>
+      </c>
+      <c r="E184" t="str">
+        <v>105070_Admin</v>
+      </c>
+      <c r="F184" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G184" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H184" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I184" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185">
+        <v>184</v>
+      </c>
+      <c r="B185" t="str">
+        <v>105062</v>
+      </c>
+      <c r="C185" t="str">
+        <v>Ban Thư ký TH</v>
+      </c>
+      <c r="D185" t="str">
+        <v>Ban Thư ký TH</v>
+      </c>
+      <c r="E185" t="str">
+        <v>105062_Admin</v>
+      </c>
+      <c r="F185" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G185" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H185" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I185" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186">
+        <v>185</v>
+      </c>
+      <c r="B186" t="str">
+        <v>105005</v>
+      </c>
+      <c r="C186" t="str">
+        <v>Văn phòng TSC</v>
+      </c>
+      <c r="D186" t="str">
+        <v>Văn phòng TSC</v>
+      </c>
+      <c r="E186" t="str">
+        <v>105005_Admin</v>
+      </c>
+      <c r="F186" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G186" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H186" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I186" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187">
+        <v>186</v>
+      </c>
+      <c r="B187" t="str">
+        <v>1020</v>
+      </c>
+      <c r="C187" t="str">
+        <v>Trung tâm CNTT</v>
+      </c>
+      <c r="D187" t="str">
+        <v>Trung tâm CNTT</v>
+      </c>
+      <c r="E187" t="str">
+        <v>1020_Admin</v>
+      </c>
+      <c r="F187" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G187" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H187" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I187" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188">
+        <v>187</v>
+      </c>
+      <c r="B188" t="str">
+        <v>105094</v>
+      </c>
+      <c r="C188" t="str">
+        <v>BQLDA ĐT XDKV</v>
+      </c>
+      <c r="D188" t="str">
+        <v>BQLDA ĐT XDKV</v>
+      </c>
+      <c r="E188" t="str">
+        <v>105094_Admin</v>
+      </c>
+      <c r="F188" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G188" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H188" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I188" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189">
+        <v>188</v>
+      </c>
+      <c r="B189" t="str">
+        <v>106000</v>
+      </c>
+      <c r="C189" t="str">
+        <v>VP Miền Trung</v>
+      </c>
+      <c r="D189" t="str">
+        <v>VP Miền Trung</v>
+      </c>
+      <c r="E189" t="str">
+        <v>106000_Admin</v>
+      </c>
+      <c r="F189" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G189" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H189" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I189" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190">
+        <v>189</v>
+      </c>
+      <c r="B190" t="str">
+        <v>105053</v>
+      </c>
+      <c r="C190" t="str">
+        <v>Ban Ngân Hàng Số</v>
+      </c>
+      <c r="D190" t="str">
+        <v>Ban Ngân Hàng Số</v>
+      </c>
+      <c r="E190" t="str">
+        <v>105053_Admin</v>
+      </c>
+      <c r="F190" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G190" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H190" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I190" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191">
+        <v>190</v>
+      </c>
+      <c r="B191" t="str">
+        <v>105020</v>
+      </c>
+      <c r="C191" t="str">
+        <v>Ban Truyền thông</v>
+      </c>
+      <c r="D191" t="str">
+        <v>Ban Truyền thông</v>
+      </c>
+      <c r="E191" t="str">
+        <v>105020_Admin</v>
+      </c>
+      <c r="F191" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G191" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H191" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I191" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192">
+        <v>191</v>
+      </c>
+      <c r="B192" t="str">
+        <v>105042</v>
+      </c>
+      <c r="C192" t="str">
+        <v>Ban Công nghệ</v>
+      </c>
+      <c r="D192" t="str">
+        <v>Ban Công nghệ</v>
+      </c>
+      <c r="E192" t="str">
+        <v>105042_Admin</v>
+      </c>
+      <c r="F192" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G192" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H192" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I192" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193">
+        <v>192</v>
+      </c>
+      <c r="B193" t="str">
+        <v>105061</v>
+      </c>
+      <c r="C193" t="str">
+        <v>BQLĐT nội ngành</v>
+      </c>
+      <c r="D193" t="str">
+        <v>BQLĐT nội ngành</v>
+      </c>
+      <c r="E193" t="str">
+        <v>105061_Admin</v>
+      </c>
+      <c r="F193" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G193" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H193" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I193" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194">
+        <v>193</v>
+      </c>
+      <c r="B194" t="str">
+        <v>105040</v>
+      </c>
+      <c r="C194" t="str">
+        <v>Ban quản lý E3</v>
+      </c>
+      <c r="D194" t="str">
+        <v>Ban quản lý E3</v>
+      </c>
+      <c r="E194" t="str">
+        <v>105040_Admin</v>
+      </c>
+      <c r="F194" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G194" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H194" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I194" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195">
+        <v>194</v>
+      </c>
+      <c r="B195" t="str">
+        <v>105084</v>
+      </c>
+      <c r="C195" t="str">
+        <v>UB Đầu tư</v>
+      </c>
+      <c r="D195" t="str">
+        <v>UB Đầu tư</v>
+      </c>
+      <c r="E195" t="str">
+        <v>105084_Admin</v>
+      </c>
+      <c r="F195" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G195" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H195" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I195" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I158"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I195"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add 11 remaining head office units and admin accounts (total 48 units)
</commit_message>
<xml_diff>
--- a/exports/Danh_sach_tai_khoan_Agribank.xlsx
+++ b/exports/Danh_sach_tai_khoan_Agribank.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I195"/>
+  <dimension ref="A1:I206"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -6065,9 +6065,328 @@
         <v>Tài khoản kê khai &amp; lập nhu cầu</v>
       </c>
     </row>
+    <row r="196">
+      <c r="A196">
+        <v>195</v>
+      </c>
+      <c r="B196" t="str">
+        <v>105014</v>
+      </c>
+      <c r="C196" t="str">
+        <v>TTTT Thương mại</v>
+      </c>
+      <c r="D196" t="str">
+        <v>TTTT Thương mại</v>
+      </c>
+      <c r="E196" t="str">
+        <v>105014_Admin</v>
+      </c>
+      <c r="F196" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G196" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H196" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I196" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197">
+        <v>196</v>
+      </c>
+      <c r="B197" t="str">
+        <v>105015</v>
+      </c>
+      <c r="C197" t="str">
+        <v>Cq Đoàn Thanh niên</v>
+      </c>
+      <c r="D197" t="str">
+        <v>Cq Đoàn Thanh niên</v>
+      </c>
+      <c r="E197" t="str">
+        <v>105015_Admin</v>
+      </c>
+      <c r="F197" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G197" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H197" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I197" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198">
+        <v>197</v>
+      </c>
+      <c r="B198" t="str">
+        <v>105055</v>
+      </c>
+      <c r="C198" t="str">
+        <v>UB Nhân sự</v>
+      </c>
+      <c r="D198" t="str">
+        <v>UB Nhân sự</v>
+      </c>
+      <c r="E198" t="str">
+        <v>105055_Admin</v>
+      </c>
+      <c r="F198" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G198" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H198" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I198" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199">
+        <v>198</v>
+      </c>
+      <c r="B199" t="str">
+        <v>105008</v>
+      </c>
+      <c r="C199" t="str">
+        <v>TT QLRR phi TD</v>
+      </c>
+      <c r="D199" t="str">
+        <v>TT QLRR phi TD</v>
+      </c>
+      <c r="E199" t="str">
+        <v>105008_Admin</v>
+      </c>
+      <c r="F199" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G199" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H199" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I199" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200">
+        <v>199</v>
+      </c>
+      <c r="B200" t="str">
+        <v>105004</v>
+      </c>
+      <c r="C200" t="str">
+        <v>Ban Pháp chế</v>
+      </c>
+      <c r="D200" t="str">
+        <v>Ban Pháp chế</v>
+      </c>
+      <c r="E200" t="str">
+        <v>105004_Admin</v>
+      </c>
+      <c r="F200" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G200" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H200" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I200" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201">
+        <v>200</v>
+      </c>
+      <c r="B201" t="str">
+        <v>105039</v>
+      </c>
+      <c r="C201" t="str">
+        <v>Ban Thư ký HĐTV</v>
+      </c>
+      <c r="D201" t="str">
+        <v>Ban Thư ký HĐTV</v>
+      </c>
+      <c r="E201" t="str">
+        <v>105039_Admin</v>
+      </c>
+      <c r="F201" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G201" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H201" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I201" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202">
+        <v>201</v>
+      </c>
+      <c r="B202" t="str">
+        <v>1010</v>
+      </c>
+      <c r="C202" t="str">
+        <v>VPĐD KV Tây Nam Bộ</v>
+      </c>
+      <c r="D202" t="str">
+        <v>VPĐD KV Tây Nam Bộ</v>
+      </c>
+      <c r="E202" t="str">
+        <v>1010_Admin</v>
+      </c>
+      <c r="F202" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G202" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H202" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I202" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203">
+        <v>202</v>
+      </c>
+      <c r="B203" t="str">
+        <v>105006</v>
+      </c>
+      <c r="C203" t="str">
+        <v>UB KT Đảng Ủy</v>
+      </c>
+      <c r="D203" t="str">
+        <v>UB KT Đảng Ủy</v>
+      </c>
+      <c r="E203" t="str">
+        <v>105006_Admin</v>
+      </c>
+      <c r="F203" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G203" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H203" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I203" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204">
+        <v>203</v>
+      </c>
+      <c r="B204" t="str">
+        <v>105016</v>
+      </c>
+      <c r="C204" t="str">
+        <v>TTPC rửa tiền</v>
+      </c>
+      <c r="D204" t="str">
+        <v>TTPC rửa tiền</v>
+      </c>
+      <c r="E204" t="str">
+        <v>105016_Admin</v>
+      </c>
+      <c r="F204" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G204" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H204" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I204" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205">
+        <v>204</v>
+      </c>
+      <c r="B205" t="str">
+        <v>105017</v>
+      </c>
+      <c r="C205" t="str">
+        <v>Ban Kiểm soát</v>
+      </c>
+      <c r="D205" t="str">
+        <v>Ban Kiểm soát</v>
+      </c>
+      <c r="E205" t="str">
+        <v>105017_Admin</v>
+      </c>
+      <c r="F205" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G205" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H205" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I205" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206">
+        <v>205</v>
+      </c>
+      <c r="B206" t="str">
+        <v>105056</v>
+      </c>
+      <c r="C206" t="str">
+        <v>Ban TC Đảng Ủy</v>
+      </c>
+      <c r="D206" t="str">
+        <v>Ban TC Đảng Ủy</v>
+      </c>
+      <c r="E206" t="str">
+        <v>105056_Admin</v>
+      </c>
+      <c r="F206" t="str">
+        <v>Unit@123456</v>
+      </c>
+      <c r="G206" t="str">
+        <v>Quản trị Đơn vị (Unit Admin)</v>
+      </c>
+      <c r="H206" t="str">
+        <v>Đang hoạt động</v>
+      </c>
+      <c r="I206" t="str">
+        <v>Tài khoản kê khai &amp; lập nhu cầu</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I195"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I206"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>